<commit_message>
Document end-to-end verification of the business plan model
Record that the workbook was validated in a real spreadsheet
application (LibreOffice Calc), not just generated: it recalculates on
open with no blank cells, reproduces all 228 printed PDF figures, and
scenario switching drives the P&L and returns correctly.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01288KGpga6FaPFxDrLS6m22
</commit_message>
<xml_diff>
--- a/business-plan/downtown-house-model.xlsx
+++ b/business-plan/downtown-house-model.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -646,151 +646,158 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (If a spreadsheet app shows zeros, force a recalculation — e.g. Ctrl+Shift+F9 in LibreOffice.)</t>
+          <t xml:space="preserve">   (Verified: the file recalculates automatically on open. If any app ever shows zeros,</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   force a recalculation — Ctrl+Shift+F9 in LibreOffice, F9 in Excel.)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>HOW THE MODEL WORKS (all proven against the PDF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>- Rooms: 5 rooms x 365 days; occupancy ramps 65/70/75/80%, flat at 80% thereafter.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- ADR ramps to the stabilised level in 2028, then grows at inflation (2%). The PDF prints ADR</t>
+          <t>- Rooms: 5 rooms x 365 days; occupancy ramps 65/70/75/80%, flat at 80% thereafter.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  rounded to whole euros; the inputs hold the exact implied values (113.22/121.90/130.88/140.50).</t>
+          <t>- ADR ramps to the stabilised level in 2028, then grows at inflation (2%). The PDF prints ADR</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>- F&amp;B revenue: direct inputs for 2025-2028, then +2% per year.</t>
+          <t xml:space="preserve">  rounded to whole euros; the inputs hold the exact implied values (113.22/121.90/130.88/140.50).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>- Departmental costs: Rooms = 12.28/11.96/11.68/11.40% of room revenue (11.40% from 2028);</t>
+          <t>- F&amp;B revenue: direct inputs for 2025-2028, then +2% per year.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  F&amp;B = 37.5% of F&amp;B revenue; Staff = EUR 533,868 in 2025 growing 2%/year (32 FTEs).</t>
+          <t>- Departmental costs: Rooms = 12.28/11.96/11.68/11.40% of room revenue (11.40% from 2028);</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>- Undistributed: A&amp;G = EUR 82,212 fixed (grows 2%/yr) + 2% of revenue; Marketing 3%;</t>
+          <t xml:space="preserve">  F&amp;B = 37.5% of F&amp;B revenue; Staff = EUR 533,868 in 2025 growing 2%/year (32 FTEs).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Property Ops &amp; Maintenance 3%; Utilities 4.5% of total revenue.</t>
+          <t>- Undistributed: A&amp;G = EUR 82,212 fixed (grows 2%/yr) + 2% of revenue; Marketing 3%;</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>- Fixed charges: rent EUR 15,000 (2024-2029), EUR 21,000 (2030-2034), EUR 90,000 from 2035;</t>
+          <t xml:space="preserve">  Property Ops &amp; Maintenance 3%; Utilities 4.5% of total revenue.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  reserve for replacement 1% of revenue in year 1, 2% thereafter.</t>
+          <t>- Fixed charges: rent EUR 15,000 (2024-2029), EUR 21,000 (2030-2034), EUR 90,000 from 2035;</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>- Returns: CAPEX EUR 1.5m + EUR 100k pre-opening, both +24% VAT paid in 2024; VAT fully</t>
+          <t xml:space="preserve">  reserve for replacement 1% of revenue in year 1, 2% thereafter.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>- Returns: CAPEX EUR 1.5m + EUR 100k pre-opening, both +24% VAT paid in 2024; VAT fully</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t xml:space="preserve">  recovered in 2025; NPV at 10% with the 2024 outflow discounted one year (Excel NPV convention).</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>CAVEATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>- The EUR 90,000 rent from 2035 is not printed anywhere in the PDF; it is the value implied by the</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PDF's 2044 NOI (414,765) and NPV (746,821). Check it against the actual lease before relying on it.</t>
+          <t>- The EUR 90,000 rent from 2035 is not printed anywhere in the PDF; it is the value implied by the</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>- The ramp-up values (ADR, F&amp;B, rooms-cost %) are taken as direct inputs; the consultants may have</t>
+          <t xml:space="preserve">  PDF's 2044 NOI (414,765) and NPV (746,821). Check it against the actual lease before relying on it.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  derived them from a monthly/seasonality model that annual figures cannot reveal.</t>
+          <t>- The ramp-up values (ADR, F&amp;B, rooms-cost %) are taken as direct inputs; the consultants may have</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>- The CAPEX grant driver (plan mentions applying for 60-75%) is set to 0% in Base, received 2025.</t>
+          <t xml:space="preserve">  derived them from a monthly/seasonality model that annual figures cannot reveal.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
+        <is>
+          <t>- The CAPEX grant driver (plan mentions applying for 60-75%) is set to 0% in Base, received 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>- This reconstruction is for analysis; it is not GBR Consulting's original file.</t>
         </is>

</xml_diff>